<commit_message>
Add Base Dados tratada + Analises + Dashboard
</commit_message>
<xml_diff>
--- a/analise/Analise de Pagamentos de E-Commerce.xlsx
+++ b/analise/Analise de Pagamentos de E-Commerce.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\us\Documents\My Docs BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586E49EF-F784-4522-9EA0-1C6AE1CB210A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB1CD00-450C-4DF9-A1B8-17E12B4A4DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="5" xr2:uid="{F192A4D9-915E-42DD-9A1C-6E8A5BFC5807}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F192A4D9-915E-42DD-9A1C-6E8A5BFC5807}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="16" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -889,7 +889,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -899,243 +899,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="82">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <sz val="18"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$USD]_-;\-* #,##0.00\ [$USD]_-;_-* &quot;-&quot;??\ [$USD]_-;_-@_-"/>
     </dxf>
@@ -1163,49 +933,28 @@
     <dxf>
       <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="18"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Novo modelo" pivot="0" table="0" count="3" xr9:uid="{32101312-6F3A-4424-93CA-7A7A88986925}">
-      <tableStyleElement type="wholeTable" dxfId="28"/>
+      <tableStyleElement type="wholeTable" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{46F421CA-312F-682f-3DD2-61675219B42D}">
-      <x14:dxfs count="4">
-        <dxf>
-          <fill>
-            <patternFill>
-              <bgColor theme="8" tint="-0.24994659260841701"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <sz val="18"/>
-            <color auto="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor theme="0"/>
-            </patternFill>
-          </fill>
-          <border>
-            <left style="thick">
-              <color auto="1"/>
-            </left>
-            <right style="thick">
-              <color auto="1"/>
-            </right>
-            <top style="thick">
-              <color auto="1"/>
-            </top>
-            <bottom style="thick">
-              <color auto="1"/>
-            </bottom>
-          </border>
-        </dxf>
+      <x14:dxfs count="2">
         <dxf>
           <fill>
             <patternFill>
@@ -1273,7 +1022,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Analise Loja Vitual.xlsx]Pagamento_por_regiao!Tabela dinâmica4</c:name>
+    <c:name>[Analise de Pagamentos de E-Commerce.xlsx]Pagamento_por_regiao!Tabela dinâmica4</c:name>
     <c:fmtId val="6"/>
   </c:pivotSource>
   <c:chart>
@@ -1928,7 +1677,7 @@
         <c:idx val="9"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent1">
+            <a:schemeClr val="accent2">
               <a:alpha val="85000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -2587,7 +2336,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Analise Loja Vitual.xlsx]Quantidade_por_meio!Tabela dinâmica4</c:name>
+    <c:name>[Analise de Pagamentos de E-Commerce.xlsx]Quantidade_por_meio!Tabela dinâmica4</c:name>
     <c:fmtId val="7"/>
   </c:pivotSource>
   <c:chart>
@@ -3302,7 +3051,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Analise Loja Vitual.xlsx]Receita_por_pagamento!Tabela dinâmica1</c:name>
+    <c:name>[Analise de Pagamentos de E-Commerce.xlsx]Receita_por_pagamento!Tabela dinâmica1</c:name>
     <c:fmtId val="10"/>
   </c:pivotSource>
   <c:chart>
@@ -3857,7 +3606,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Analise Loja Vitual.xlsx]Categoria_por_Meio!Tabela dinâmica5</c:name>
+    <c:name>[Analise de Pagamentos de E-Commerce.xlsx]Categoria_por_Meio!Tabela dinâmica5</c:name>
     <c:fmtId val="4"/>
   </c:pivotSource>
   <c:chart>
@@ -6887,8 +6636,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="11" name="Meses">
@@ -6911,7 +6660,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -7163,7 +6912,7 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:fld id="{314F9160-0E0F-4929-9A69-D34E748DF2FC}" type="TxLink">
+          <a:fld id="{7170710F-0856-4F7B-AF89-678AFA47B4F3}" type="TxLink">
             <a:rPr lang="en-US" sz="2400" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
@@ -7171,7 +6920,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:t> 51 170,86 USD </a:t>
+            <a:t> 80 567,85 USD </a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2400" b="1"/>
         </a:p>
@@ -11091,7 +10840,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{810B1823-2DA4-41E9-AC98-E5CED2804122}" name="Tabela dinâmica1" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{810B1823-2DA4-41E9-AC98-E5CED2804122}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -11528,7 +11277,7 @@
     <dataField name="Soma de Total Revenue" fld="7" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="74">
+    <format dxfId="1">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -11583,7 +11332,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36934170-3729-411B-833A-B5F881521992}" name="Tabela dinâmica4" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36934170-3729-411B-833A-B5F881521992}" name="Tabela dinâmica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="A11:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -11682,7 +11431,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AE2C46B1-3DE6-42A3-A57E-0B75D962DF4F}" name="Tabela dinâmica4" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AE2C46B1-3DE6-42A3-A57E-0B75D962DF4F}" name="Tabela dinâmica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A3:E8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -12205,62 +11954,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{42A9D4A4-15AE-4230-95A5-AFF21A8C24FD}" name="Tabela dinâmica3" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B15:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="12">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="14">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma de Total Revenue" fld="7" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5A012574-60B8-4C9D-AA71-709C66122C0F}" name="Tabela dinâmica5" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5A012574-60B8-4C9D-AA71-709C66122C0F}" name="Tabela dinâmica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A3:E11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -12730,7 +12424,7 @@
     <dataField name="Soma de Total Revenue" fld="7" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="73">
+    <format dxfId="0">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -12772,6 +12466,61 @@
       </pivotArea>
     </chartFormat>
   </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{42A9D4A4-15AE-4230-95A5-AFF21A8C24FD}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B15:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma de Total Revenue" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -12849,29 +12598,23 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A1603CB-D84B-435F-AB2A-9C2BC684F027}" name="Online_Sales_Data" displayName="Online_Sales_Data" ref="A1:K241" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:K241" xr:uid="{9A1603CB-D84B-435F-AB2A-9C2BC684F027}">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="Credit Card"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K241" xr:uid="{9A1603CB-D84B-435F-AB2A-9C2BC684F027}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{BC45A562-9AE0-42DF-99BC-67B8848D1806}" uniqueName="1" name="Transaction ID" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{A9E77E48-121D-4002-BE19-E65AAF11EB66}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="81"/>
-    <tableColumn id="3" xr3:uid="{D10D8704-AD80-414D-B6C6-78C07DF6893E}" uniqueName="3" name="Product Category" queryTableFieldId="3" dataDxfId="80"/>
-    <tableColumn id="4" xr3:uid="{54F209B8-C9ED-4167-B8B1-95A037252847}" uniqueName="4" name="Product Name" queryTableFieldId="4" dataDxfId="79"/>
+    <tableColumn id="2" xr3:uid="{A9E77E48-121D-4002-BE19-E65AAF11EB66}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{D10D8704-AD80-414D-B6C6-78C07DF6893E}" uniqueName="3" name="Product Category" queryTableFieldId="3" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{54F209B8-C9ED-4167-B8B1-95A037252847}" uniqueName="4" name="Product Name" queryTableFieldId="4" dataDxfId="6"/>
     <tableColumn id="5" xr3:uid="{10F65675-D5A7-4C8C-BFF0-09B25C219167}" uniqueName="5" name="Units Sold" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{49FF1127-2FA3-4D85-A524-F886AFF84DCE}" uniqueName="6" name="Unit Price" queryTableFieldId="6"/>
-    <tableColumn id="10" xr3:uid="{5437880E-5AA2-4EF1-A51F-94177AEC9184}" uniqueName="10" name="Expected Revenue" queryTableFieldId="10" dataDxfId="78">
+    <tableColumn id="10" xr3:uid="{5437880E-5AA2-4EF1-A51F-94177AEC9184}" uniqueName="10" name="Expected Revenue" queryTableFieldId="10" dataDxfId="5">
       <calculatedColumnFormula>Online_Sales_Data[[#This Row],[Units Sold]]*Online_Sales_Data[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{B094CCA8-32FE-469F-B562-DE596935BC84}" uniqueName="7" name="Total Revenue" queryTableFieldId="7"/>
-    <tableColumn id="11" xr3:uid="{A37F74C0-9356-44DF-BCED-F9EB664B20E8}" uniqueName="11" name="Discount" queryTableFieldId="11" dataDxfId="77">
+    <tableColumn id="11" xr3:uid="{A37F74C0-9356-44DF-BCED-F9EB664B20E8}" uniqueName="11" name="Discount" queryTableFieldId="11" dataDxfId="4">
       <calculatedColumnFormula>Online_Sales_Data[[#This Row],[Expected Revenue]]-Online_Sales_Data[[#This Row],[Total Revenue]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{04B751FB-1FE5-4A95-AD3F-D46720BE1F38}" uniqueName="8" name="Region" queryTableFieldId="8" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{F9E5A4E3-7ADF-42FE-96BA-B5697F3632C2}" uniqueName="9" name="Payment Method" queryTableFieldId="9" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{04B751FB-1FE5-4A95-AD3F-D46720BE1F38}" uniqueName="8" name="Region" queryTableFieldId="8" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{F9E5A4E3-7ADF-42FE-96BA-B5697F3632C2}" uniqueName="9" name="Payment Method" queryTableFieldId="9" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -13262,7 +13005,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10002</v>
       </c>
@@ -13299,7 +13042,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>10003</v>
       </c>
@@ -13373,7 +13116,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>10005</v>
       </c>
@@ -13484,7 +13227,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>10008</v>
       </c>
@@ -13521,7 +13264,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10009</v>
       </c>
@@ -13595,7 +13338,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10011</v>
       </c>
@@ -13706,7 +13449,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>10014</v>
       </c>
@@ -13743,7 +13486,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>10015</v>
       </c>
@@ -13817,7 +13560,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>10017</v>
       </c>
@@ -13928,7 +13671,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>10020</v>
       </c>
@@ -13965,7 +13708,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>10021</v>
       </c>
@@ -14039,7 +13782,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>10023</v>
       </c>
@@ -14150,7 +13893,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>10026</v>
       </c>
@@ -14187,7 +13930,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>10027</v>
       </c>
@@ -14261,7 +14004,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>10029</v>
       </c>
@@ -14372,7 +14115,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>10032</v>
       </c>
@@ -14409,7 +14152,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>10033</v>
       </c>
@@ -14483,7 +14226,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>10035</v>
       </c>
@@ -14594,7 +14337,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>10038</v>
       </c>
@@ -14631,7 +14374,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>10039</v>
       </c>
@@ -14705,7 +14448,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>10041</v>
       </c>
@@ -14816,7 +14559,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>10044</v>
       </c>
@@ -14853,7 +14596,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>10045</v>
       </c>
@@ -14927,7 +14670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>10047</v>
       </c>
@@ -15038,7 +14781,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>10050</v>
       </c>
@@ -15075,7 +14818,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>10051</v>
       </c>
@@ -15149,7 +14892,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>10053</v>
       </c>
@@ -15260,7 +15003,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>10056</v>
       </c>
@@ -15297,7 +15040,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>10057</v>
       </c>
@@ -15371,7 +15114,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>10059</v>
       </c>
@@ -15482,7 +15225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>10062</v>
       </c>
@@ -15519,7 +15262,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>10063</v>
       </c>
@@ -15593,7 +15336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>10065</v>
       </c>
@@ -15704,7 +15447,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>10068</v>
       </c>
@@ -15741,7 +15484,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>10069</v>
       </c>
@@ -15815,7 +15558,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>10071</v>
       </c>
@@ -15926,7 +15669,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>10074</v>
       </c>
@@ -15963,7 +15706,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>10075</v>
       </c>
@@ -16037,7 +15780,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>10077</v>
       </c>
@@ -16148,7 +15891,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>10080</v>
       </c>
@@ -16185,7 +15928,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>10081</v>
       </c>
@@ -16259,7 +16002,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>10083</v>
       </c>
@@ -16370,7 +16113,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>10086</v>
       </c>
@@ -16407,7 +16150,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>10087</v>
       </c>
@@ -16481,7 +16224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>10089</v>
       </c>
@@ -16592,7 +16335,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>10092</v>
       </c>
@@ -16629,7 +16372,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>10093</v>
       </c>
@@ -16703,7 +16446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>10095</v>
       </c>
@@ -16814,7 +16557,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>10098</v>
       </c>
@@ -16851,7 +16594,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>10099</v>
       </c>
@@ -16925,7 +16668,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>10101</v>
       </c>
@@ -17036,7 +16779,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>10104</v>
       </c>
@@ -17073,7 +16816,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>10105</v>
       </c>
@@ -17147,7 +16890,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>10107</v>
       </c>
@@ -17258,7 +17001,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>10110</v>
       </c>
@@ -17295,7 +17038,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>10111</v>
       </c>
@@ -17369,7 +17112,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>10113</v>
       </c>
@@ -17480,7 +17223,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>10116</v>
       </c>
@@ -17517,7 +17260,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>10117</v>
       </c>
@@ -17591,7 +17334,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>10119</v>
       </c>
@@ -17702,7 +17445,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>10122</v>
       </c>
@@ -17739,7 +17482,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="124" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>10123</v>
       </c>
@@ -17813,7 +17556,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>10125</v>
       </c>
@@ -17924,7 +17667,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="129" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>10128</v>
       </c>
@@ -17961,7 +17704,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="130" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>10129</v>
       </c>
@@ -18035,7 +17778,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="132" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>10131</v>
       </c>
@@ -18146,7 +17889,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="135" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>10134</v>
       </c>
@@ -18183,7 +17926,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>10135</v>
       </c>
@@ -18257,7 +18000,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="138" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>10137</v>
       </c>
@@ -18368,7 +18111,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="141" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>10140</v>
       </c>
@@ -18405,7 +18148,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="142" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>10141</v>
       </c>
@@ -18479,7 +18222,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="144" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>10143</v>
       </c>
@@ -18590,7 +18333,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="147" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>10146</v>
       </c>
@@ -18627,7 +18370,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="148" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>10147</v>
       </c>
@@ -18701,7 +18444,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="150" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>10149</v>
       </c>
@@ -18812,7 +18555,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="153" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>10152</v>
       </c>
@@ -18849,7 +18592,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>10153</v>
       </c>
@@ -18923,7 +18666,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="156" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>10155</v>
       </c>
@@ -19034,7 +18777,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="159" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>10158</v>
       </c>
@@ -19071,7 +18814,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="160" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>10159</v>
       </c>
@@ -19145,7 +18888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="162" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>10161</v>
       </c>
@@ -19256,7 +18999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="165" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>10164</v>
       </c>
@@ -19293,7 +19036,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>10165</v>
       </c>
@@ -19367,7 +19110,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="168" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>10167</v>
       </c>
@@ -19478,7 +19221,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="171" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>10170</v>
       </c>
@@ -19515,7 +19258,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="172" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>10171</v>
       </c>
@@ -19589,7 +19332,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="174" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>10173</v>
       </c>
@@ -19700,7 +19443,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="177" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>10176</v>
       </c>
@@ -19737,7 +19480,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="178" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>10177</v>
       </c>
@@ -19811,7 +19554,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="180" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>10179</v>
       </c>
@@ -19922,7 +19665,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="183" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>10182</v>
       </c>
@@ -19959,7 +19702,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="184" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>10183</v>
       </c>
@@ -20033,7 +19776,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="186" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>10185</v>
       </c>
@@ -20144,7 +19887,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="189" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>10188</v>
       </c>
@@ -20181,7 +19924,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="190" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>10189</v>
       </c>
@@ -20255,7 +19998,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="192" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>10191</v>
       </c>
@@ -20366,7 +20109,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="195" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>10194</v>
       </c>
@@ -20403,7 +20146,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="196" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>10195</v>
       </c>
@@ -20477,7 +20220,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="198" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>10197</v>
       </c>
@@ -20588,7 +20331,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="201" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>10200</v>
       </c>
@@ -20625,7 +20368,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="202" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>10201</v>
       </c>
@@ -20699,7 +20442,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="204" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>10203</v>
       </c>
@@ -20810,7 +20553,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="207" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>10206</v>
       </c>
@@ -20847,7 +20590,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="208" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>10207</v>
       </c>
@@ -20921,7 +20664,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="210" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>10209</v>
       </c>
@@ -21032,7 +20775,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="213" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>10212</v>
       </c>
@@ -21069,7 +20812,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="214" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>10213</v>
       </c>
@@ -21143,7 +20886,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="216" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>10215</v>
       </c>
@@ -21254,7 +20997,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="219" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>10218</v>
       </c>
@@ -21291,7 +21034,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="220" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>10219</v>
       </c>
@@ -21365,7 +21108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="222" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>10221</v>
       </c>
@@ -21476,7 +21219,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="225" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>10224</v>
       </c>
@@ -21513,7 +21256,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="226" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>10225</v>
       </c>
@@ -21587,7 +21330,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="228" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>10227</v>
       </c>
@@ -21698,7 +21441,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="231" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>10230</v>
       </c>
@@ -21735,7 +21478,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="232" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>10231</v>
       </c>
@@ -21809,7 +21552,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="234" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>10233</v>
       </c>
@@ -21920,7 +21663,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="237" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>10236</v>
       </c>
@@ -21957,7 +21700,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="238" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>10237</v>
       </c>
@@ -22031,7 +21774,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="240" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>10239</v>
       </c>
@@ -22189,7 +21932,7 @@
       <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12">
         <v>120</v>
       </c>
     </row>
@@ -22197,7 +21940,7 @@
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13">
         <v>40</v>
       </c>
     </row>
@@ -22205,7 +21948,7 @@
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14">
         <v>80</v>
       </c>
     </row>
@@ -22213,7 +21956,7 @@
       <c r="A15" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15">
         <v>240</v>
       </c>
     </row>
@@ -22341,8 +22084,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.88671875" bestFit="1" customWidth="1"/>
@@ -22477,11 +22219,11 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="7">
+      <c r="B16">
         <v>80567.850000000079</v>
       </c>
-      <c r="C16" s="8">
-        <v>51170.86</v>
+      <c r="C16" s="7">
+        <v>80567.850000000006</v>
       </c>
       <c r="E16">
         <v>0</v>

</xml_diff>